<commit_message>
Handle sin templo in citizen support
</commit_message>
<xml_diff>
--- a/data/Gestion apoyo ciudadano Kennedy.xlsx
+++ b/data/Gestion apoyo ciudadano Kennedy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernandozamora/Documents/Kennedy/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656C0C6B-B64A-784C-8DD6-5706BD75A6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8464D5-086D-2445-8294-4B8F9BE974C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1560" yWindow="2080" windowWidth="26840" windowHeight="15160" xr2:uid="{05F58CEF-06E0-6F43-9C75-43722292F70E}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3681" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3681" uniqueCount="552">
   <si>
     <t>Lorena Garzon</t>
   </si>
@@ -1748,6 +1748,9 @@
   </si>
   <si>
     <t>Corporación</t>
+  </si>
+  <si>
+    <t>08.Sin Templo</t>
   </si>
 </sst>
 </file>
@@ -2132,6 +2135,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26C9F862-44FC-7C41-B3A1-4BF7AAA19378}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:P346"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
@@ -2182,7 +2186,7 @@
         <v>536</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>154</v>
       </c>
@@ -2229,7 +2233,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>154</v>
       </c>
@@ -2276,7 +2280,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>154</v>
       </c>
@@ -2321,7 +2325,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>154</v>
       </c>
@@ -2368,7 +2372,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>154</v>
       </c>
@@ -2413,7 +2417,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>154</v>
       </c>
@@ -2458,7 +2462,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>154</v>
       </c>
@@ -2505,7 +2509,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>154</v>
       </c>
@@ -2552,7 +2556,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>154</v>
       </c>
@@ -2599,7 +2603,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
         <v>154</v>
       </c>
@@ -2646,7 +2650,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
         <v>154</v>
       </c>
@@ -2693,7 +2697,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
         <v>154</v>
       </c>
@@ -2740,7 +2744,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
         <v>154</v>
       </c>
@@ -2785,7 +2789,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
         <v>154</v>
       </c>
@@ -2832,7 +2836,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
         <v>154</v>
       </c>
@@ -2879,7 +2883,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
         <v>154</v>
       </c>
@@ -2926,7 +2930,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
         <v>154</v>
       </c>
@@ -2971,7 +2975,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
         <v>154</v>
       </c>
@@ -3016,7 +3020,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
         <v>154</v>
       </c>
@@ -3063,7 +3067,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
         <v>154</v>
       </c>
@@ -3110,7 +3114,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
         <v>154</v>
       </c>
@@ -3157,7 +3161,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="23" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
         <v>154</v>
       </c>
@@ -3204,7 +3208,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="24" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
         <v>154</v>
       </c>
@@ -3249,7 +3253,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="25" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
         <v>154</v>
       </c>
@@ -3296,7 +3300,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="26" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
         <v>154</v>
       </c>
@@ -3343,7 +3347,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="27" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
         <v>154</v>
       </c>
@@ -3390,7 +3394,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="28" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
         <v>154</v>
       </c>
@@ -3435,7 +3439,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="29" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
         <v>154</v>
       </c>
@@ -3480,7 +3484,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="30" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
         <v>154</v>
       </c>
@@ -3525,7 +3529,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="31" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
         <v>154</v>
       </c>
@@ -3572,7 +3576,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="32" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
         <v>154</v>
       </c>
@@ -3617,7 +3621,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="33" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
         <v>154</v>
       </c>
@@ -3662,7 +3666,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="34" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
         <v>154</v>
       </c>
@@ -3709,7 +3713,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="35" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
         <v>154</v>
       </c>
@@ -3754,7 +3758,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="36" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
         <v>154</v>
       </c>
@@ -3799,7 +3803,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="37" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
         <v>154</v>
       </c>
@@ -3844,7 +3848,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="38" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
         <v>154</v>
       </c>
@@ -3891,7 +3895,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="39" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A39" t="s">
         <v>154</v>
       </c>
@@ -3936,7 +3940,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="40" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
         <v>154</v>
       </c>
@@ -3981,7 +3985,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="41" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
         <v>154</v>
       </c>
@@ -4026,7 +4030,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="42" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A42" t="s">
         <v>154</v>
       </c>
@@ -4073,7 +4077,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="43" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A43" t="s">
         <v>154</v>
       </c>
@@ -4118,7 +4122,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="44" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A44" t="s">
         <v>154</v>
       </c>
@@ -4165,7 +4169,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="45" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A45" t="s">
         <v>154</v>
       </c>
@@ -4212,7 +4216,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="46" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A46" t="s">
         <v>154</v>
       </c>
@@ -4259,7 +4263,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="47" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A47" t="s">
         <v>154</v>
       </c>
@@ -4304,7 +4308,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="48" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A48" t="s">
         <v>154</v>
       </c>
@@ -4349,7 +4353,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="49" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A49" t="s">
         <v>154</v>
       </c>
@@ -4396,7 +4400,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="50" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
         <v>154</v>
       </c>
@@ -4443,7 +4447,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="51" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A51" t="s">
         <v>154</v>
       </c>
@@ -4488,7 +4492,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="52" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A52" t="s">
         <v>154</v>
       </c>
@@ -4533,7 +4537,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="53" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A53" t="s">
         <v>154</v>
       </c>
@@ -4578,7 +4582,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="54" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A54" t="s">
         <v>154</v>
       </c>
@@ -4623,7 +4627,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="55" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A55" t="s">
         <v>154</v>
       </c>
@@ -4668,7 +4672,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="56" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A56" t="s">
         <v>154</v>
       </c>
@@ -4713,7 +4717,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="57" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A57" t="s">
         <v>154</v>
       </c>
@@ -4756,7 +4760,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="58" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A58" t="s">
         <v>154</v>
       </c>
@@ -4801,7 +4805,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="59" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A59" t="s">
         <v>154</v>
       </c>
@@ -4846,7 +4850,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="60" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A60" t="s">
         <v>154</v>
       </c>
@@ -4893,7 +4897,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="61" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A61" t="s">
         <v>154</v>
       </c>
@@ -4940,7 +4944,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="62" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A62" t="s">
         <v>154</v>
       </c>
@@ -4985,7 +4989,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="63" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A63" t="s">
         <v>154</v>
       </c>
@@ -5032,7 +5036,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="64" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A64" t="s">
         <v>154</v>
       </c>
@@ -5079,7 +5083,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="65" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A65" t="s">
         <v>154</v>
       </c>
@@ -5126,7 +5130,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="66" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A66" t="s">
         <v>154</v>
       </c>
@@ -5171,7 +5175,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="67" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A67" t="s">
         <v>154</v>
       </c>
@@ -5218,7 +5222,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="68" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A68" t="s">
         <v>154</v>
       </c>
@@ -5263,7 +5267,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="69" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A69" t="s">
         <v>154</v>
       </c>
@@ -5310,7 +5314,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="70" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A70" t="s">
         <v>154</v>
       </c>
@@ -5353,7 +5357,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="71" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A71" t="s">
         <v>154</v>
       </c>
@@ -5400,7 +5404,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="72" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A72" t="s">
         <v>154</v>
       </c>
@@ -5447,7 +5451,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="73" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A73" t="s">
         <v>154</v>
       </c>
@@ -5494,7 +5498,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="74" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A74" t="s">
         <v>154</v>
       </c>
@@ -5539,7 +5543,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="75" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A75" t="s">
         <v>154</v>
       </c>
@@ -5586,7 +5590,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="76" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A76" t="s">
         <v>154</v>
       </c>
@@ -5631,7 +5635,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="77" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A77" t="s">
         <v>154</v>
       </c>
@@ -5676,7 +5680,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="78" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A78" t="s">
         <v>154</v>
       </c>
@@ -5721,7 +5725,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="79" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A79" t="s">
         <v>154</v>
       </c>
@@ -5766,7 +5770,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="80" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A80" t="s">
         <v>154</v>
       </c>
@@ -5809,7 +5813,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="81" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A81" t="s">
         <v>154</v>
       </c>
@@ -5852,7 +5856,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="82" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A82" t="s">
         <v>154</v>
       </c>
@@ -5897,7 +5901,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="83" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A83" t="s">
         <v>154</v>
       </c>
@@ -5944,7 +5948,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="84" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A84" t="s">
         <v>154</v>
       </c>
@@ -5989,7 +5993,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="85" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A85" t="s">
         <v>154</v>
       </c>
@@ -6036,7 +6040,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="86" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A86" t="s">
         <v>154</v>
       </c>
@@ -6083,7 +6087,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="87" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -6130,7 +6134,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="88" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A88" t="s">
         <v>154</v>
       </c>
@@ -6177,7 +6181,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="89" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A89" t="s">
         <v>154</v>
       </c>
@@ -6224,7 +6228,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="90" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A90" t="s">
         <v>154</v>
       </c>
@@ -6271,7 +6275,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="91" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A91" t="s">
         <v>154</v>
       </c>
@@ -6318,7 +6322,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="92" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A92" t="s">
         <v>154</v>
       </c>
@@ -6365,7 +6369,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="93" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A93" t="s">
         <v>154</v>
       </c>
@@ -6412,7 +6416,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="94" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A94" t="s">
         <v>154</v>
       </c>
@@ -6459,7 +6463,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="95" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A95" t="s">
         <v>154</v>
       </c>
@@ -6504,7 +6508,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="96" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A96" t="s">
         <v>154</v>
       </c>
@@ -6551,7 +6555,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="97" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A97" t="s">
         <v>154</v>
       </c>
@@ -6598,7 +6602,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="98" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A98" t="s">
         <v>154</v>
       </c>
@@ -6645,7 +6649,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="99" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A99" t="s">
         <v>154</v>
       </c>
@@ -6692,7 +6696,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="100" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A100" t="s">
         <v>154</v>
       </c>
@@ -6739,7 +6743,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="101" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A101" t="s">
         <v>154</v>
       </c>
@@ -6786,7 +6790,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="102" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A102" t="s">
         <v>154</v>
       </c>
@@ -6833,7 +6837,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="103" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A103" t="s">
         <v>154</v>
       </c>
@@ -6880,7 +6884,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="104" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A104" t="s">
         <v>154</v>
       </c>
@@ -6927,7 +6931,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="105" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A105" t="s">
         <v>154</v>
       </c>
@@ -6974,7 +6978,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="106" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A106" t="s">
         <v>154</v>
       </c>
@@ -7021,7 +7025,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="107" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A107" t="s">
         <v>154</v>
       </c>
@@ -7068,7 +7072,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="108" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A108" t="s">
         <v>154</v>
       </c>
@@ -7115,7 +7119,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="109" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A109" t="s">
         <v>154</v>
       </c>
@@ -7162,7 +7166,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="110" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A110" t="s">
         <v>154</v>
       </c>
@@ -7209,7 +7213,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A111" t="s">
         <v>154</v>
       </c>
@@ -7256,7 +7260,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A112" t="s">
         <v>154</v>
       </c>
@@ -7303,7 +7307,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="113" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A113" t="s">
         <v>154</v>
       </c>
@@ -7350,7 +7354,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="114" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A114" t="s">
         <v>154</v>
       </c>
@@ -7397,7 +7401,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="115" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A115" t="s">
         <v>154</v>
       </c>
@@ -7444,7 +7448,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="116" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A116" t="s">
         <v>154</v>
       </c>
@@ -7491,7 +7495,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="117" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A117" t="s">
         <v>154</v>
       </c>
@@ -7536,7 +7540,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="118" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A118" t="s">
         <v>154</v>
       </c>
@@ -7583,7 +7587,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="119" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A119" t="s">
         <v>154</v>
       </c>
@@ -7630,7 +7634,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="120" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A120" t="s">
         <v>154</v>
       </c>
@@ -7677,7 +7681,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="121" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A121" t="s">
         <v>154</v>
       </c>
@@ -7724,7 +7728,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="122" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A122" t="s">
         <v>154</v>
       </c>
@@ -7771,7 +7775,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="123" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A123" t="s">
         <v>154</v>
       </c>
@@ -7818,7 +7822,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="124" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A124" t="s">
         <v>154</v>
       </c>
@@ -7865,7 +7869,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="125" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A125" t="s">
         <v>154</v>
       </c>
@@ -7912,7 +7916,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="126" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A126" t="s">
         <v>154</v>
       </c>
@@ -7959,7 +7963,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="127" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="127" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A127" t="s">
         <v>154</v>
       </c>
@@ -8006,7 +8010,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="128" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="128" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A128" t="s">
         <v>154</v>
       </c>
@@ -8053,7 +8057,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="129" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A129" t="s">
         <v>154</v>
       </c>
@@ -8100,7 +8104,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="130" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A130" t="s">
         <v>154</v>
       </c>
@@ -8147,7 +8151,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="131" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A131" t="s">
         <v>154</v>
       </c>
@@ -8194,7 +8198,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="132" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A132" t="s">
         <v>154</v>
       </c>
@@ -8241,7 +8245,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A133" t="s">
         <v>154</v>
       </c>
@@ -8288,7 +8292,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="134" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A134" t="s">
         <v>154</v>
       </c>
@@ -8335,7 +8339,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="135" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A135" t="s">
         <v>154</v>
       </c>
@@ -8382,7 +8386,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="136" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A136" t="s">
         <v>154</v>
       </c>
@@ -8429,7 +8433,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="137" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A137" t="s">
         <v>154</v>
       </c>
@@ -8476,7 +8480,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="138" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A138" t="s">
         <v>154</v>
       </c>
@@ -8523,7 +8527,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="139" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A139" t="s">
         <v>154</v>
       </c>
@@ -8570,7 +8574,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="140" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A140" t="s">
         <v>154</v>
       </c>
@@ -8617,7 +8621,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="141" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A141" t="s">
         <v>154</v>
       </c>
@@ -8664,7 +8668,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="142" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A142" t="s">
         <v>154</v>
       </c>
@@ -8711,7 +8715,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="143" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A143" t="s">
         <v>154</v>
       </c>
@@ -8758,7 +8762,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="144" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A144" t="s">
         <v>154</v>
       </c>
@@ -8805,7 +8809,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="145" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="145" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A145" t="s">
         <v>154</v>
       </c>
@@ -8852,7 +8856,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="146" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="146" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A146" t="s">
         <v>154</v>
       </c>
@@ -8899,7 +8903,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="147" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="147" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A147" t="s">
         <v>154</v>
       </c>
@@ -8946,7 +8950,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="148" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="148" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A148" t="s">
         <v>154</v>
       </c>
@@ -8993,7 +8997,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="149" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="149" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A149" t="s">
         <v>154</v>
       </c>
@@ -9040,7 +9044,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="150" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="150" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A150" t="s">
         <v>154</v>
       </c>
@@ -9087,7 +9091,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="151" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="151" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A151" t="s">
         <v>154</v>
       </c>
@@ -9134,7 +9138,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="152" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="152" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A152" t="s">
         <v>154</v>
       </c>
@@ -9173,7 +9177,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="153" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="153" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A153" t="s">
         <v>154</v>
       </c>
@@ -9212,7 +9216,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="154" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="154" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A154" t="s">
         <v>154</v>
       </c>
@@ -9251,7 +9255,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="155" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="155" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A155" t="s">
         <v>154</v>
       </c>
@@ -9298,7 +9302,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="156" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="156" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A156" t="s">
         <v>154</v>
       </c>
@@ -9339,7 +9343,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="157" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="157" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A157" t="s">
         <v>154</v>
       </c>
@@ -9380,7 +9384,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="158" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="158" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A158" t="s">
         <v>154</v>
       </c>
@@ -9421,7 +9425,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="159" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="159" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A159" t="s">
         <v>154</v>
       </c>
@@ -9462,7 +9466,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="160" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="160" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A160" t="s">
         <v>154</v>
       </c>
@@ -9503,7 +9507,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="161" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="161" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A161" t="s">
         <v>154</v>
       </c>
@@ -9544,7 +9548,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="162" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="162" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A162" t="s">
         <v>154</v>
       </c>
@@ -9585,7 +9589,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="163" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="163" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A163" t="s">
         <v>154</v>
       </c>
@@ -9624,7 +9628,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="164" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="164" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A164" t="s">
         <v>154</v>
       </c>
@@ -9665,7 +9669,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="165" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="165" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A165" t="s">
         <v>154</v>
       </c>
@@ -9704,7 +9708,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="166" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="166" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A166" t="s">
         <v>154</v>
       </c>
@@ -9743,7 +9747,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="167" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="167" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A167" t="s">
         <v>154</v>
       </c>
@@ -9782,7 +9786,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="168" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="168" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A168" t="s">
         <v>154</v>
       </c>
@@ -9821,7 +9825,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="169" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="169" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A169" t="s">
         <v>154</v>
       </c>
@@ -9868,7 +9872,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="170" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="170" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A170" t="s">
         <v>154</v>
       </c>
@@ -9915,7 +9919,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="171" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="171" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A171" t="s">
         <v>154</v>
       </c>
@@ -9954,7 +9958,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="172" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="172" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A172" t="s">
         <v>154</v>
       </c>
@@ -9993,7 +9997,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="173" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="173" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A173" t="s">
         <v>154</v>
       </c>
@@ -10032,7 +10036,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="174" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="174" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A174" t="s">
         <v>154</v>
       </c>
@@ -10073,7 +10077,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="175" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="175" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A175" t="s">
         <v>154</v>
       </c>
@@ -10114,7 +10118,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="176" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="176" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A176" t="s">
         <v>154</v>
       </c>
@@ -10154,7 +10158,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="177" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="177" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A177" t="s">
         <v>154</v>
       </c>
@@ -10195,7 +10199,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="178" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="178" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A178" t="s">
         <v>154</v>
       </c>
@@ -10242,7 +10246,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="179" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="179" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A179" t="s">
         <v>154</v>
       </c>
@@ -10289,7 +10293,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="180" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="180" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A180" t="s">
         <v>154</v>
       </c>
@@ -10336,7 +10340,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="181" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="181" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A181" t="s">
         <v>154</v>
       </c>
@@ -10383,7 +10387,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="182" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="182" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A182" t="s">
         <v>154</v>
       </c>
@@ -10430,7 +10434,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="183" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="183" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A183" t="s">
         <v>154</v>
       </c>
@@ -10477,7 +10481,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="184" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="184" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A184" t="s">
         <v>154</v>
       </c>
@@ -10524,7 +10528,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="185" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="185" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A185" t="s">
         <v>154</v>
       </c>
@@ -10571,7 +10575,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="186" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="186" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A186" t="s">
         <v>154</v>
       </c>
@@ -10618,7 +10622,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="187" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="187" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A187" t="s">
         <v>154</v>
       </c>
@@ -10665,7 +10669,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="188" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="188" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A188" t="s">
         <v>154</v>
       </c>
@@ -10712,7 +10716,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="189" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="189" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A189" t="s">
         <v>154</v>
       </c>
@@ -10759,7 +10763,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="190" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="190" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A190" t="s">
         <v>154</v>
       </c>
@@ -10806,7 +10810,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="191" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="191" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A191" t="s">
         <v>154</v>
       </c>
@@ -10853,7 +10857,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="192" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="192" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A192" t="s">
         <v>154</v>
       </c>
@@ -10900,7 +10904,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="193" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="193" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A193" t="s">
         <v>154</v>
       </c>
@@ -10947,7 +10951,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="194" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="194" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A194" t="s">
         <v>154</v>
       </c>
@@ -10994,7 +10998,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="195" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="195" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A195" t="s">
         <v>154</v>
       </c>
@@ -11041,7 +11045,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="196" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="196" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A196" t="s">
         <v>154</v>
       </c>
@@ -11088,7 +11092,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="197" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="197" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A197" t="s">
         <v>154</v>
       </c>
@@ -11127,7 +11131,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="198" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="198" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A198" t="s">
         <v>154</v>
       </c>
@@ -11166,7 +11170,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="199" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="199" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A199" t="s">
         <v>154</v>
       </c>
@@ -11205,7 +11209,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="200" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="200" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A200" t="s">
         <v>154</v>
       </c>
@@ -11244,7 +11248,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="201" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="201" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A201" t="s">
         <v>154</v>
       </c>
@@ -11283,7 +11287,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="202" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="202" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A202" t="s">
         <v>154</v>
       </c>
@@ -11322,7 +11326,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="203" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="203" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A203" t="s">
         <v>154</v>
       </c>
@@ -11363,7 +11367,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="204" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="204" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A204" t="s">
         <v>154</v>
       </c>
@@ -11410,7 +11414,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="205" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="205" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A205" t="s">
         <v>154</v>
       </c>
@@ -11457,7 +11461,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="206" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="206" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A206" t="s">
         <v>154</v>
       </c>
@@ -11504,7 +11508,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="207" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="207" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A207" t="s">
         <v>154</v>
       </c>
@@ -11551,7 +11555,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="208" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="208" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A208" t="s">
         <v>154</v>
       </c>
@@ -11598,7 +11602,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="209" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="209" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A209" t="s">
         <v>154</v>
       </c>
@@ -11645,7 +11649,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="210" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="210" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A210" t="s">
         <v>154</v>
       </c>
@@ -11692,7 +11696,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="211" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="211" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A211" t="s">
         <v>154</v>
       </c>
@@ -11739,7 +11743,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="212" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="212" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A212" t="s">
         <v>154</v>
       </c>
@@ -11786,7 +11790,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="213" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="213" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A213" t="s">
         <v>154</v>
       </c>
@@ -11833,7 +11837,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="214" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="214" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A214" t="s">
         <v>154</v>
       </c>
@@ -11876,7 +11880,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="215" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="215" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A215" t="s">
         <v>154</v>
       </c>
@@ -11919,7 +11923,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="216" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="216" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A216" t="s">
         <v>154</v>
       </c>
@@ -11962,7 +11966,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="217" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="217" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A217" t="s">
         <v>154</v>
       </c>
@@ -12005,7 +12009,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="218" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="218" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A218" t="s">
         <v>154</v>
       </c>
@@ -12048,7 +12052,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="219" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="219" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A219" t="s">
         <v>154</v>
       </c>
@@ -12087,7 +12091,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="220" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="220" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A220" t="s">
         <v>154</v>
       </c>
@@ -12130,7 +12134,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="221" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="221" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A221" t="s">
         <v>154</v>
       </c>
@@ -12177,7 +12181,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="222" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="222" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A222" t="s">
         <v>154</v>
       </c>
@@ -12224,7 +12228,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="223" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="223" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A223" t="s">
         <v>154</v>
       </c>
@@ -12271,7 +12275,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="224" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="224" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A224" t="s">
         <v>154</v>
       </c>
@@ -12318,7 +12322,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="225" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="225" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A225" t="s">
         <v>154</v>
       </c>
@@ -12365,7 +12369,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="226" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="226" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A226" t="s">
         <v>154</v>
       </c>
@@ -12412,7 +12416,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="227" spans="1:16" ht="126" x14ac:dyDescent="0.15">
+    <row r="227" spans="1:16" ht="126" hidden="1" x14ac:dyDescent="0.15">
       <c r="A227" t="s">
         <v>154</v>
       </c>
@@ -12459,7 +12463,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="228" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="228" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A228" t="s">
         <v>154</v>
       </c>
@@ -12506,7 +12510,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="229" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="229" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A229" t="s">
         <v>154</v>
       </c>
@@ -12553,7 +12557,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="230" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="230" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A230" t="s">
         <v>154</v>
       </c>
@@ -12600,7 +12604,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="231" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="231" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A231" t="s">
         <v>154</v>
       </c>
@@ -12647,7 +12651,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="232" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="232" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A232" t="s">
         <v>154</v>
       </c>
@@ -12687,7 +12691,7 @@
       </c>
       <c r="P232" s="2"/>
     </row>
-    <row r="233" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="233" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A233" t="s">
         <v>154</v>
       </c>
@@ -12729,7 +12733,7 @@
       </c>
       <c r="P233" s="2"/>
     </row>
-    <row r="234" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="234" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A234" t="s">
         <v>154</v>
       </c>
@@ -12769,7 +12773,7 @@
       </c>
       <c r="P234" s="2"/>
     </row>
-    <row r="235" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="235" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A235" t="s">
         <v>154</v>
       </c>
@@ -12809,7 +12813,7 @@
       </c>
       <c r="P235" s="2"/>
     </row>
-    <row r="236" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="236" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A236" t="s">
         <v>154</v>
       </c>
@@ -12849,7 +12853,7 @@
       </c>
       <c r="P236" s="2"/>
     </row>
-    <row r="237" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="237" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A237" t="s">
         <v>154</v>
       </c>
@@ -12889,7 +12893,7 @@
       </c>
       <c r="P237" s="2"/>
     </row>
-    <row r="238" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="238" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A238" t="s">
         <v>154</v>
       </c>
@@ -12929,7 +12933,7 @@
       </c>
       <c r="P238" s="2"/>
     </row>
-    <row r="239" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="239" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A239" t="s">
         <v>154</v>
       </c>
@@ -12969,7 +12973,7 @@
       </c>
       <c r="P239" s="2"/>
     </row>
-    <row r="240" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="240" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A240" t="s">
         <v>154</v>
       </c>
@@ -13011,7 +13015,7 @@
       </c>
       <c r="P240" s="2"/>
     </row>
-    <row r="241" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="241" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A241" t="s">
         <v>154</v>
       </c>
@@ -13053,7 +13057,7 @@
       </c>
       <c r="P241" s="2"/>
     </row>
-    <row r="242" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="242" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A242" t="s">
         <v>154</v>
       </c>
@@ -13095,7 +13099,7 @@
       </c>
       <c r="P242" s="2"/>
     </row>
-    <row r="243" spans="1:16" ht="14" x14ac:dyDescent="0.15">
+    <row r="243" spans="1:16" ht="14" hidden="1" x14ac:dyDescent="0.15">
       <c r="A243" t="s">
         <v>154</v>
       </c>
@@ -13137,7 +13141,7 @@
       </c>
       <c r="P243" s="2"/>
     </row>
-    <row r="244" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="244" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A244" t="s">
         <v>5</v>
       </c>
@@ -13178,7 +13182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="245" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A245" t="s">
         <v>5</v>
       </c>
@@ -13219,7 +13223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="246" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A246" t="s">
         <v>5</v>
       </c>
@@ -13260,7 +13264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="247" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A247" t="s">
         <v>5</v>
       </c>
@@ -13301,7 +13305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="248" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A248" t="s">
         <v>5</v>
       </c>
@@ -13342,7 +13346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="249" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A249" t="s">
         <v>5</v>
       </c>
@@ -13383,7 +13387,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="250" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A250" t="s">
         <v>5</v>
       </c>
@@ -13424,7 +13428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="251" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A251" t="s">
         <v>5</v>
       </c>
@@ -13465,7 +13469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="252" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A252" t="s">
         <v>5</v>
       </c>
@@ -13506,7 +13510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="253" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A253" t="s">
         <v>5</v>
       </c>
@@ -13547,7 +13551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="254" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A254" t="s">
         <v>5</v>
       </c>
@@ -13588,7 +13592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="255" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A255" t="s">
         <v>5</v>
       </c>
@@ -13629,7 +13633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:16" x14ac:dyDescent="0.15">
+    <row r="256" spans="1:16" hidden="1" x14ac:dyDescent="0.15">
       <c r="A256" t="s">
         <v>5</v>
       </c>
@@ -13670,7 +13674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="257" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A257" t="s">
         <v>5</v>
       </c>
@@ -13711,7 +13715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="258" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A258" t="s">
         <v>5</v>
       </c>
@@ -13752,7 +13756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="259" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A259" t="s">
         <v>5</v>
       </c>
@@ -13793,7 +13797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="260" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A260" t="s">
         <v>5</v>
       </c>
@@ -13834,7 +13838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="261" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A261" t="s">
         <v>5</v>
       </c>
@@ -13875,7 +13879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="262" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A262" t="s">
         <v>5</v>
       </c>
@@ -13916,7 +13920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="263" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A263" t="s">
         <v>5</v>
       </c>
@@ -13957,7 +13961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="264" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A264" t="s">
         <v>5</v>
       </c>
@@ -13998,7 +14002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="265" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A265" t="s">
         <v>5</v>
       </c>
@@ -14039,7 +14043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="266" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A266" t="s">
         <v>5</v>
       </c>
@@ -14080,7 +14084,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="267" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A267" t="s">
         <v>5</v>
       </c>
@@ -14121,7 +14125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="268" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A268" t="s">
         <v>5</v>
       </c>
@@ -14162,7 +14166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="269" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A269" t="s">
         <v>5</v>
       </c>
@@ -14203,7 +14207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="270" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A270" t="s">
         <v>5</v>
       </c>
@@ -14244,7 +14248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="271" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A271" t="s">
         <v>5</v>
       </c>
@@ -14285,7 +14289,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="272" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="272" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A272" t="s">
         <v>5</v>
       </c>
@@ -14326,7 +14330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="273" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A273" t="s">
         <v>5</v>
       </c>
@@ -14367,7 +14371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="274" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A274" t="s">
         <v>5</v>
       </c>
@@ -14408,7 +14412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="275" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A275" t="s">
         <v>5</v>
       </c>
@@ -14449,7 +14453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="276" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="276" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A276" t="s">
         <v>5</v>
       </c>
@@ -14490,7 +14494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="277" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="277" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A277" t="s">
         <v>5</v>
       </c>
@@ -14531,7 +14535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="278" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="278" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A278" t="s">
         <v>5</v>
       </c>
@@ -14572,7 +14576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="279" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="279" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A279" t="s">
         <v>5</v>
       </c>
@@ -14613,7 +14617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="280" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A280" t="s">
         <v>5</v>
       </c>
@@ -14654,7 +14658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="281" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A281" t="s">
         <v>5</v>
       </c>
@@ -14695,7 +14699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="282" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A282" t="s">
         <v>5</v>
       </c>
@@ -14736,7 +14740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="283" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A283" t="s">
         <v>5</v>
       </c>
@@ -14777,7 +14781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="284" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A284" t="s">
         <v>5</v>
       </c>
@@ -14818,7 +14822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="285" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A285" t="s">
         <v>5</v>
       </c>
@@ -14859,7 +14863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="286" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A286" t="s">
         <v>5</v>
       </c>
@@ -14900,7 +14904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="287" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="287" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A287" t="s">
         <v>5</v>
       </c>
@@ -14941,7 +14945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="288" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A288" t="s">
         <v>5</v>
       </c>
@@ -14982,7 +14986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="289" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A289" t="s">
         <v>5</v>
       </c>
@@ -15023,7 +15027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="290" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A290" t="s">
         <v>5</v>
       </c>
@@ -15064,7 +15068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="291" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A291" t="s">
         <v>5</v>
       </c>
@@ -15105,7 +15109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="292" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A292" t="s">
         <v>5</v>
       </c>
@@ -15146,7 +15150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="293" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A293" t="s">
         <v>5</v>
       </c>
@@ -15187,7 +15191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="294" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="294" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A294" t="s">
         <v>5</v>
       </c>
@@ -15228,7 +15232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="295" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A295" t="s">
         <v>5</v>
       </c>
@@ -15269,7 +15273,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="296" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="296" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A296" t="s">
         <v>5</v>
       </c>
@@ -15310,7 +15314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="297" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="297" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A297" t="s">
         <v>5</v>
       </c>
@@ -15351,7 +15355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="298" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A298" t="s">
         <v>5</v>
       </c>
@@ -15392,7 +15396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="299" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A299" t="s">
         <v>5</v>
       </c>
@@ -15433,7 +15437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="300" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A300" t="s">
         <v>5</v>
       </c>
@@ -15474,7 +15478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="301" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A301" t="s">
         <v>5</v>
       </c>
@@ -15515,7 +15519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="302" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="302" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A302" t="s">
         <v>5</v>
       </c>
@@ -15556,7 +15560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="303" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="303" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A303" t="s">
         <v>5</v>
       </c>
@@ -15597,7 +15601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="304" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="304" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A304" t="s">
         <v>5</v>
       </c>
@@ -15638,7 +15642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="305" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A305" t="s">
         <v>5</v>
       </c>
@@ -15679,7 +15683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="306" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="306" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A306" t="s">
         <v>5</v>
       </c>
@@ -15720,7 +15724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="307" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="307" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A307" t="s">
         <v>5</v>
       </c>
@@ -15761,7 +15765,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="308" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A308" t="s">
         <v>5</v>
       </c>
@@ -15802,7 +15806,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="309" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A309" t="s">
         <v>5</v>
       </c>
@@ -15843,7 +15847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="310" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A310" t="s">
         <v>5</v>
       </c>
@@ -15884,7 +15888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="311" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A311" t="s">
         <v>5</v>
       </c>
@@ -15925,7 +15929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="312" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A312" t="s">
         <v>5</v>
       </c>
@@ -15966,7 +15970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="313" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A313" t="s">
         <v>5</v>
       </c>
@@ -16007,7 +16011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="314" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A314" t="s">
         <v>5</v>
       </c>
@@ -16048,7 +16052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="315" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A315" t="s">
         <v>5</v>
       </c>
@@ -16089,7 +16093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="316" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A316" t="s">
         <v>5</v>
       </c>
@@ -16130,7 +16134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="317" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A317" t="s">
         <v>5</v>
       </c>
@@ -16171,7 +16175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="318" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A318" t="s">
         <v>5</v>
       </c>
@@ -16212,7 +16216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="319" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A319" t="s">
         <v>5</v>
       </c>
@@ -16253,7 +16257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="320" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A320" t="s">
         <v>5</v>
       </c>
@@ -16294,7 +16298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="321" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A321" t="s">
         <v>5</v>
       </c>
@@ -16335,7 +16339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="322" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A322" t="s">
         <v>5</v>
       </c>
@@ -16373,7 +16377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="323" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="323" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A323" t="s">
         <v>5</v>
       </c>
@@ -16413,7 +16417,7 @@
         <v>5</v>
       </c>
       <c r="L324" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O324" t="s">
         <v>0</v>
@@ -16448,13 +16452,13 @@
         <v>14</v>
       </c>
       <c r="L325" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O325" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="326" spans="1:15" ht="112" x14ac:dyDescent="0.15">
+    <row r="326" spans="1:15" ht="112" hidden="1" x14ac:dyDescent="0.15">
       <c r="A326" t="s">
         <v>5</v>
       </c>
@@ -16495,7 +16499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="327" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A327" t="s">
         <v>5</v>
       </c>
@@ -16565,7 +16569,7 @@
         <v>14</v>
       </c>
       <c r="L328" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O328" t="s">
         <v>0</v>
@@ -16597,7 +16601,7 @@
         <v>45</v>
       </c>
       <c r="L329" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O329" t="s">
         <v>0</v>
@@ -16629,7 +16633,7 @@
         <v>43</v>
       </c>
       <c r="L330" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O330" t="s">
         <v>0</v>
@@ -16661,7 +16665,7 @@
         <v>42</v>
       </c>
       <c r="L331" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O331" t="s">
         <v>0</v>
@@ -16693,13 +16697,13 @@
         <v>41</v>
       </c>
       <c r="L332" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O332" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="333" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A333" t="s">
         <v>5</v>
       </c>
@@ -16740,7 +16744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="334" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="334" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A334" t="s">
         <v>5</v>
       </c>
@@ -16804,7 +16808,7 @@
         <v>36</v>
       </c>
       <c r="L335" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O335" t="s">
         <v>0</v>
@@ -16836,7 +16840,7 @@
         <v>33</v>
       </c>
       <c r="L336" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O336" t="s">
         <v>0</v>
@@ -16868,7 +16872,7 @@
         <v>30</v>
       </c>
       <c r="L337" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O337" t="s">
         <v>0</v>
@@ -16897,13 +16901,13 @@
         <v>29</v>
       </c>
       <c r="L338" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O338" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="339" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A339" t="s">
         <v>5</v>
       </c>
@@ -16970,7 +16974,7 @@
         <v>23</v>
       </c>
       <c r="L340" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O340" t="s">
         <v>0</v>
@@ -17002,13 +17006,13 @@
         <v>20</v>
       </c>
       <c r="L341" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O341" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="342" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="342" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A342" t="s">
         <v>5</v>
       </c>
@@ -17049,7 +17053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="343" spans="1:15" x14ac:dyDescent="0.15">
+    <row r="343" spans="1:15" hidden="1" x14ac:dyDescent="0.15">
       <c r="A343" t="s">
         <v>5</v>
       </c>
@@ -17116,7 +17120,7 @@
         <v>7</v>
       </c>
       <c r="L344" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O344" t="s">
         <v>0</v>
@@ -17148,7 +17152,7 @@
         <v>6</v>
       </c>
       <c r="L345" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O345" t="s">
         <v>0</v>
@@ -17180,14 +17184,26 @@
         <v>1</v>
       </c>
       <c r="L346" t="s">
-        <v>18</v>
+        <v>551</v>
       </c>
       <c r="O346" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:O346" xr:uid="{83A8DDE0-E41C-394B-BBBE-838851EA5B38}"/>
+  <autoFilter ref="B1:O346" xr:uid="{83A8DDE0-E41C-394B-BBBE-838851EA5B38}">
+    <filterColumn colId="7">
+      <filters blank="1"/>
+    </filterColumn>
+    <filterColumn colId="10">
+      <filters>
+        <filter val="08.Kennedy Central"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="12">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="19">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="M98:M139 M141:M142 M144:M154 M156:M175 M177:M243" xr:uid="{762315C2-0AC6-F64C-9B89-45C7CBB18B72}">
       <formula1>"En Proceso,Pendiente,Finalizado,N/A"</formula1>

</xml_diff>